<commit_message>
Support bilingual trend links and HTML import
</commit_message>
<xml_diff>
--- a/tools/trends/templates/trend-table-import-template.xlsx
+++ b/tools/trends/templates/trend-table-import-template.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,22 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F2937"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +55,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,254 +425,314 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO1"/>
+  <dimension ref="A1:AY1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
-    <col width="10" customWidth="1" min="20" max="20"/>
-    <col width="10" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
-    <col width="12" customWidth="1" min="25" max="25"/>
-    <col width="11" customWidth="1" min="26" max="26"/>
-    <col width="11" customWidth="1" min="27" max="27"/>
-    <col width="12" customWidth="1" min="28" max="28"/>
-    <col width="11" customWidth="1" min="29" max="29"/>
-    <col width="11" customWidth="1" min="30" max="30"/>
-    <col width="12" customWidth="1" min="31" max="31"/>
-    <col width="11" customWidth="1" min="32" max="32"/>
-    <col width="11" customWidth="1" min="33" max="33"/>
-    <col width="12" customWidth="1" min="34" max="34"/>
-    <col width="11" customWidth="1" min="35" max="35"/>
-    <col width="11" customWidth="1" min="36" max="36"/>
-    <col width="12" customWidth="1" min="37" max="37"/>
-    <col width="11" customWidth="1" min="38" max="38"/>
-    <col width="11" customWidth="1" min="39" max="39"/>
-    <col width="12" customWidth="1" min="40" max="40"/>
-    <col width="10" customWidth="1" min="41" max="41"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="26" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="26" customWidth="1" min="21" max="21"/>
+    <col width="26" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
+    <col width="26" customWidth="1" min="25" max="25"/>
+    <col width="26" customWidth="1" min="26" max="26"/>
+    <col width="22" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="26" customWidth="1" min="29" max="29"/>
+    <col width="26" customWidth="1" min="30" max="30"/>
+    <col width="22" customWidth="1" min="31" max="31"/>
+    <col width="22" customWidth="1" min="32" max="32"/>
+    <col width="26" customWidth="1" min="33" max="33"/>
+    <col width="26" customWidth="1" min="34" max="34"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
+    <col width="22" customWidth="1" min="36" max="36"/>
+    <col width="26" customWidth="1" min="37" max="37"/>
+    <col width="26" customWidth="1" min="38" max="38"/>
+    <col width="22" customWidth="1" min="39" max="39"/>
+    <col width="22" customWidth="1" min="40" max="40"/>
+    <col width="26" customWidth="1" min="41" max="41"/>
+    <col width="26" customWidth="1" min="42" max="42"/>
+    <col width="22" customWidth="1" min="43" max="43"/>
+    <col width="22" customWidth="1" min="44" max="44"/>
+    <col width="26" customWidth="1" min="45" max="45"/>
+    <col width="26" customWidth="1" min="46" max="46"/>
+    <col width="22" customWidth="1" min="47" max="47"/>
+    <col width="22" customWidth="1" min="48" max="48"/>
+    <col width="26" customWidth="1" min="49" max="49"/>
+    <col width="26" customWidth="1" min="50" max="50"/>
+    <col width="22" customWidth="1" min="51" max="51"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Icon URL</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Title ZH</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Title EN</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Sub ZH</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Sub EN</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Trend Intro ZH</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Trend Intro EN</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Keywords ZH</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Keywords EN</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Zone1 ZH</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Zone1 EN</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Zone1 URL</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Zone1 URL ZH</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Zone1 URL EN</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Zone2 ZH</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Zone2 EN</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Zone2 URL</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Zone2 URL ZH</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Zone2 URL EN</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Zone3 ZH</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Zone3 EN</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>Zone3 URL</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Zone3 URL ZH</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Zone3 URL EN</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Zone4 ZH</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Zone4 EN</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>Zone4 URL</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Zone4 URL ZH</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Zone4 URL EN</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Forum1 ZH</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Forum1 EN</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>Forum1 URL</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Forum1 URL ZH</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Forum1 URL EN</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Forum2 ZH</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Forum2 EN</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>Forum2 URL</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Forum2 URL ZH</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Forum2 URL EN</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Forum3 ZH</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Forum3 EN</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>Forum3 URL</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>Forum3 URL ZH</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>Forum3 URL EN</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>Forum4 ZH</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Forum4 EN</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>Forum4 URL</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>Forum4 URL ZH</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>Forum4 URL EN</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>Forum5 ZH</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>Forum5 EN</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>Forum5 URL</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>Forum5 URL ZH</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>Forum5 URL EN</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>Forum6 ZH</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>Forum6 EN</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
-        <is>
-          <t>Forum6 URL</t>
-        </is>
-      </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>Forum6 URL ZH</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>Forum6 URL EN</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>

</xml_diff>

<commit_message>
feat(trends): support grouped bilingual imports
</commit_message>
<xml_diff>
--- a/tools/trends/templates/trend-table-import-template.xlsx
+++ b/tools/trends/templates/trend-table-import-template.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trend Import Template" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Trend Import Template'!$A$1:$BB$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -27,7 +29,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F2937"/>
+      <color rgb="00222222"/>
     </font>
   </fonts>
   <fills count="3">
@@ -39,7 +41,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9EAF7"/>
+        <fgColor rgb="00E9D7EF"/>
       </patternFill>
     </fill>
   </fills>
@@ -425,60 +427,63 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY1"/>
+  <dimension ref="A1:BB1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="26" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="26" customWidth="1" min="17" max="17"/>
-    <col width="26" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
-    <col width="26" customWidth="1" min="21" max="21"/>
-    <col width="26" customWidth="1" min="22" max="22"/>
-    <col width="22" customWidth="1" min="23" max="23"/>
-    <col width="22" customWidth="1" min="24" max="24"/>
-    <col width="26" customWidth="1" min="25" max="25"/>
-    <col width="26" customWidth="1" min="26" max="26"/>
-    <col width="22" customWidth="1" min="27" max="27"/>
-    <col width="22" customWidth="1" min="28" max="28"/>
-    <col width="26" customWidth="1" min="29" max="29"/>
-    <col width="26" customWidth="1" min="30" max="30"/>
-    <col width="22" customWidth="1" min="31" max="31"/>
-    <col width="22" customWidth="1" min="32" max="32"/>
-    <col width="26" customWidth="1" min="33" max="33"/>
-    <col width="26" customWidth="1" min="34" max="34"/>
-    <col width="22" customWidth="1" min="35" max="35"/>
-    <col width="22" customWidth="1" min="36" max="36"/>
-    <col width="26" customWidth="1" min="37" max="37"/>
-    <col width="26" customWidth="1" min="38" max="38"/>
-    <col width="22" customWidth="1" min="39" max="39"/>
-    <col width="22" customWidth="1" min="40" max="40"/>
-    <col width="26" customWidth="1" min="41" max="41"/>
-    <col width="26" customWidth="1" min="42" max="42"/>
-    <col width="22" customWidth="1" min="43" max="43"/>
-    <col width="22" customWidth="1" min="44" max="44"/>
-    <col width="26" customWidth="1" min="45" max="45"/>
-    <col width="26" customWidth="1" min="46" max="46"/>
-    <col width="22" customWidth="1" min="47" max="47"/>
-    <col width="22" customWidth="1" min="48" max="48"/>
-    <col width="26" customWidth="1" min="49" max="49"/>
-    <col width="26" customWidth="1" min="50" max="50"/>
-    <col width="22" customWidth="1" min="51" max="51"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
+    <col width="24" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="24" customWidth="1" min="24" max="24"/>
+    <col width="24" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="24" customWidth="1" min="28" max="28"/>
+    <col width="24" customWidth="1" min="29" max="29"/>
+    <col width="14" customWidth="1" min="30" max="30"/>
+    <col width="14" customWidth="1" min="31" max="31"/>
+    <col width="24" customWidth="1" min="32" max="32"/>
+    <col width="24" customWidth="1" min="33" max="33"/>
+    <col width="14" customWidth="1" min="34" max="34"/>
+    <col width="14" customWidth="1" min="35" max="35"/>
+    <col width="24" customWidth="1" min="36" max="36"/>
+    <col width="24" customWidth="1" min="37" max="37"/>
+    <col width="14" customWidth="1" min="38" max="38"/>
+    <col width="14" customWidth="1" min="39" max="39"/>
+    <col width="24" customWidth="1" min="40" max="40"/>
+    <col width="24" customWidth="1" min="41" max="41"/>
+    <col width="14" customWidth="1" min="42" max="42"/>
+    <col width="14" customWidth="1" min="43" max="43"/>
+    <col width="24" customWidth="1" min="44" max="44"/>
+    <col width="24" customWidth="1" min="45" max="45"/>
+    <col width="14" customWidth="1" min="46" max="46"/>
+    <col width="14" customWidth="1" min="47" max="47"/>
+    <col width="24" customWidth="1" min="48" max="48"/>
+    <col width="24" customWidth="1" min="49" max="49"/>
+    <col width="14" customWidth="1" min="50" max="50"/>
+    <col width="14" customWidth="1" min="51" max="51"/>
+    <col width="24" customWidth="1" min="52" max="52"/>
+    <col width="24" customWidth="1" min="53" max="53"/>
+    <col width="32" customWidth="1" min="54" max="54"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -534,211 +539,227 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Group ZH</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Group EN</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Zone1 ZH</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Zone1 EN</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Zone1 URL ZH</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Zone1 URL EN</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Zone2 ZH</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Zone2 EN</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Zone2 URL ZH</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Zone2 URL EN</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Zone3 ZH</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Zone3 EN</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Zone3 URL ZH</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Zone3 URL EN</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Zone4 ZH</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Zone4 EN</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Zone4 URL ZH</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Zone4 URL EN</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Forum1 ZH</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Forum1 EN</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Forum1 URL ZH</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Forum1 URL EN</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Forum2 ZH</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Forum2 EN</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Forum2 URL ZH</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Forum2 URL EN</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Forum3 ZH</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>Forum3 EN</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Forum3 URL ZH</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>Forum3 URL EN</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>Forum4 ZH</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>Forum4 EN</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>Forum4 URL ZH</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>Forum4 URL EN</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>Forum5 ZH</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>Forum5 EN</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>Forum5 URL ZH</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>Forum5 URL EN</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>Forum6 ZH</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>Forum6 EN</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>Forum6 URL ZH</t>
         </is>
       </c>
-      <c r="AX1" s="1" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>Forum6 URL EN</t>
         </is>
       </c>
-      <c r="AY1" s="1" t="inlineStr">
+      <c r="BB1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:BB1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>